<commit_message>
chore: job feed run 2026-10-25 18:46 UTC
</commit_message>
<xml_diff>
--- a/output/DataEngineerJobs_2026-10-26.xlsx
+++ b/output/DataEngineerJobs_2026-10-26.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Run Log" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Jobs'!$A$1:$P$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Jobs'!$A$1:$P$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Excluded'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,10 +33,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <color rgb="001155CC"/>
-      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -64,16 +60,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -440,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -543,123 +533,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>SoFi</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Senior Data Engineer</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Cottonwood Heights, Utah, United States</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>unspecified</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Full-time</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>https://sofi.com/careers/job/8040823003?gh_jid=8040823003</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>https://sofi.com/careers/job/8040823003?gh_jid=8040823003</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>5yr</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-24 02:37</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>greenhouse</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>open (live company feed)</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>Employee Applicant Privacy Notice
-Who we are:
-Shape a brighter financial future with us.
-Together with our members, we’re changing the way people think about and interact with personal finance.
-We’re a next-generation financial services company and national bank using innovative, mobile-first technology to help our millions of members reach their goals. The industry is going through an unprecedented transformation, and we’re at the forefront. We’re proud to come to work every day knowing that what we do has a direct impact on people’s lives, with our core values guiding us every step of the way. Join us to invest in yourself, your career, and the financial world.
-The Role: 
-SoFi's Fraud Prevention Center of Excellence (CoE) is responsible for managing enterprise fraud threats across banking products and member-related activities. The Fraud Operations Analytics &amp; Reporting team sits at the center of this mission — driving intelligence through data to improve operational efficiency, agent accountability, and fraud detection efficacy across all fraud product lines.
-We are looking for a Senior Data Engineer to build and scale the data infrastructure that powers the Fraud CoE. This role is the foundational engineering resource for the Fraud Operations Analytics team, responsible for consolidating data pipelines into governed, source-of-truth data marts and enabling the analytical work that drives operational decisions at the highest levels of the organization.
-Key Responsibilities
-Data Infrastructure &amp; Pipeline Development
-- Design, build, and maintain scalable data pipelines that consolidate fraud operational data from multiple source systems into governed Snowflake data marts
-- Partner with Fraud Data Engineering and the TDM platform team on the foundational Fraud CoE data buildout, including summarized metric tables that standardize reporting across all fraud product lines
-Data Modeling &amp; Warehouse Optimization
-- Model analytical data within Snowflake to support fraud operations reporting, agent performance scorecards, and fraud tagging quality monitoring
-- Build and maintain dbt models that structure data for easy consumption by analysts and Tableau reporting layers
-- Ensure query performance, data freshness, and reliability across all fraud data mart tables powering production dashboards and leadership reports
-Analytics Enablement
-- Partner closely with fraud analysts to understand data requirements and translate them into robust, reusable data structures
-- Develop and maintain summarized metric tables that lock reporting logic centrally, ensuring consistency across reporting
-Governance &amp; Standards
-- Establish and enforce data engineering standards, documentation practices, and pipeline design patterns for the Fraud CoE
-- Ensure all data assets are properly documented, tested, and governed to support audit and compliance requirements
-- Serve as the data engineering subject matter expert in cross-functional discussions with Fraud Strategy, Fraud Platform, Risk Infrastructure, and Data Engineering partners
-What We're Looking For
-Required
-- 4+ years of data engineering experience with strong hands-on expertise in SQL, Python, and cloud data warehouse platforms 
-- Proven experience building and maintaining production-grade data pipelines using modern data stack tools (dbt, Airflow, or equivalent)
-- Strong data modeling skills — experience designing analytical data structures optimized for reporting and self-service consumption
-- Ability to work closely with analytics and business stakeholders to translate requirements into scalable data solutions
-- Strong documentation habits and commitment to data quality, testing, and pipeline reliability
-- Exposure to dbt Cloud, Airflow/MWAA, or similar orchestration platforms
-Strongly Preferred
-- Experience in financial services, fraud, risk, or compliance data environments
-- Familiarity with fraud operations data concepts — fraud tagging, loss attribution, dispute workflows, agent performance metrics, or alert queue management
-Compensation and Benefits
-The base pay range for this role is listed below. Final base pay offer will be determined based on individual factors such as the candidate’s experience, skills, and location. 
-To view all of our comprehensive and competitive benefits, visit our Benefits at SoFi page!
-SoFi provides equal employment opportunities (EEO) to all employees and applicants for employment without regard to race, color, religion (including religious dress and grooming practices), sex (including pregnancy, childbirth and related medical conditions, breastfeeding, and conditions related to breastfeeding), gender, gender identity, gender expression, national origin, ancestry, age (40 or over), physical or medical disability, medical condition, marital status, registered domestic partner status, sexual orientation, genetic information, military and/or veteran status, or any other basis prohibited by applicable state or federal law.
-The Company hires the best qualified candidate for the job, without regard to protected characteristics.
-Pursuant to the San Francisco Fair Chance Ordinance, we will consider for employment qualified applicants with arrest and conviction records.
-New York applicants: Notice of Employee Rights
-SoFi is committed to an inclusive culture. As part of this commitment, SoFi offers reasonable accommodations to candidates with physical or mental disabilities. If you need accommodations to participate in the job application or interview process, please let your recruiter know or email accommodations@sofi.com.
-We are unable to accommodate remote work from Hawaii, Alaska or Puerto Rico at this time.
-Internal Employees
-If you are a current employee, do not apply here - please navigate to our Internal Job Board in Greenhouse to apply to our open roles.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:P2"/>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
-  </hyperlinks>
+  <autoFilter ref="A1:P1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -752,7 +627,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-25 18:43:39</t>
+          <t>2026-10-25 18:45:39</t>
         </is>
       </c>
     </row>
@@ -764,7 +639,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-26 00:13:39</t>
+          <t>2026-10-26 00:15:39</t>
         </is>
       </c>
     </row>
@@ -824,7 +699,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -848,7 +723,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: job feed run 2026-10-25 22:23 UTC
</commit_message>
<xml_diff>
--- a/output/DataEngineerJobs_2026-10-26.xlsx
+++ b/output/DataEngineerJobs_2026-10-26.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Run Log" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Jobs'!$A$1:$P$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Jobs'!$A$1:$P$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Excluded'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +33,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="001155CC"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -60,10 +64,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -430,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -533,8 +543,245 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Samsara</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Senior AI Data &amp; Analytics Engineer II</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Remote - Seattle</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>remote</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.samsara.com/company/careers/roles/8302004?gh_jid=8302004</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>accessibleinterviewing@samsara.com</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.samsara.com/company/careers/roles/8302004?gh_jid=8302004</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>5yr</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 02:25</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>open (live company feed)</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Who we are
+Samsara (NYSE: IOT) is the pioneer of the Connected Operations™ Cloud, which is a platform that enables organizations that depend on physical operations to harness Internet of Things (IoT) data to develop actionable insights and improve their operations. At Samsara, we are helping improve the safety, efficiency and sustainability of the physical operations that power our global economy. Representing more than 40% of global GDP, these industries are the infrastructure of our planet, including agriculture, construction, field services, transportation, and manufacturing — and we are excited to help digitally transform their operations at scale.
+Working at Samsara means you’ll help define the future of physical operations and be on a team that’s shaping an exciting array of product solutions, including Video-Based Safety, Vehicle Telematics, Apps and Driver Workflows, and Equipment Monitoring. As part of a recently public company, you’ll have the autonomy and support to make an impact as we build for the long term.
+About the role:
+Want to build the data foundation powering AI and self-serve analytics at scale? As part of Samsara's Marketing Data and Analytics (MDA) Engineering team, you will shape the technical roadmap alongside our BI and Data Science peers. You will architect core Databricks pipelines, Gold Layer tables, and semantic models, turning ambitious, ambiguous business challenges into high-value data products, autonomous agents, and cross-functional automation.
+This role is open to candidates residing in the US.
+You should apply if:
+- You want to impact the industries that run our world: Your efforts will result in real-world impact – helping to keep the lights on, get food into grocery stores, reduce emissions, and most importantly, ensure workers return home safely.
+- You are the architect of your own career: If you put in the work, this role won’t be your last at Samsara. We set up our employees for success and have built a culture that encourages rapid career development, countless opportunities to experiment and master your craft in a hyper growth environment.
+- You’re energized by our opportunity: The vision we have to digitize large sectors of the global economy requires your full focus and best efforts to bring forth creative, ambitious ideas for our customers.
+- You want to be with the best: At Samsara, we win together, celebrate together and support each other. You will be surrounded by a high-calibre team that will encourage you to do your best. 
+In this role, you will:
+- Partner on defining the strategy and multi-quarter roadmap for MDA's data and AI foundation.
+- Architect and own Samsara's marketing data infrastructure: ETL/ELT pipelines, Databricks Gold Layer tables, and the core data models that power segmentation, targeting, automation, and analytics.
+- Design the semantic layers, data dictionaries, and structured documentation that enable self-serve BI and conversational analytics, partnering with the BI team to ensure core sales and marketing KPIs are built on trusted, well-modeled data.
+- Translate ambiguous business questions from Marketing, Sales, and R&amp;D into clear requirements and scalable solutions, working autonomously without dedicated PM support and influencing decisions with data and sound reasoning.
+- Lead complex, cross-team initiatives end to end: stand up new data pipelines and integrations quickly, manage risk across interdependent teams, and own the reliability and data quality of what ships.
+- Serve as the senior technical lead for the team's hardest problems: raise the bar for engineering quality and code review, remove bottlenecks that slow multiple teams, and mentor engineers and analysts. 
+- Drive the strategic use of AI to solve ambiguous, high-impact problems: build AI-enabled data products and agents, with the integrations, retrieval pipelines, and evaluation practices that keep them reliable and trustworthy.
+- Identify and automate manual workflows with AI across Marketing and GTM teams, taking ideas from concept to prototype to production and influencing org roadmaps.
+- Ship high-quality Python and SQL, increasingly by directing agentic coding tools, while holding a high bar for reviewing and verifying AI-generated work before it reaches production.
+- Champion, role model, and embed Samsara’s cultural principles (Focus on Customer Success, Build for the Long Term, Adopt a Growth Mindset, Be Inclusive, Win as a Team) as we scale globally and across new offices.
+Minimum requirements for the role:
+- 8+ years of experience in data engineering, analytics engineering, or AI engineering, including deep hands-on data engineering experience.
+- Expert-level Python and SQL, with strong hands-on data modeling and DBT experience.
+- Deep experience with data warehouse and lakehouse architectures, ETL/ELT, and the modern data stack, including hands-on Databricks (or similar, such as Snowflake or BigQuery).
+- Experience building semantic layers and structured documentation optimized for AI ingestion and agentic workflows.
+- Agentic coding tools (e.g., Claude Code, Cursor) are part of your regular workflow, and you verify and take ownership of AI-generated output.
+- Experience building, shipping, evaluating, and monitoring LLM or agent systems in production.
+- Track record of leading complex, cross-team data initiatives, including independent requirements gathering with technical and non-technical stakeholders.
+- Experience supporting Marketing, Sales, or Product teams.
+An ideal candidate also has:
+- Experience working with Databricks and building AI Agents within the ecosystem. 
+- Software engineering background beyond data or AI engineering, with a track record of turning ambiguous, unfamiliar problems into well-architected, delivered solutions.
+- Expertise in data visualization and building dashboards for sales and marketing KPIs.
+- Familiarity with go-to-market data and systems: CRM (e.g., Salesforce), marketing automation, web analytics, and MarTech tools.
+- Experience building interactive applications with Streamlit, Claude workflows, or web frameworks.
+- Data science, machine learning, or predictive analytics experience.
+- Comfort working in an exploratory environment, testing and iterating on new data sources and methodologies.
+The compensation range shown spans approved pay zones for this role. Your primary work location determines the range applicable to you, which may be narrower than the full range displayed.
+The range of annual base salary for full-time employees for this position is below. Please note that base pay offered may vary depending on factors including your city of residence, job-related knowledge, skills, and experience. This role is also eligible for an initial RSU grant with no vesting cliff, and ongoing refresh opportunities tied to performance, subject to plan terms and conditions. Learn more about our total rewards and benefits below.
+Annual Base Salary
+$137,445—$231,000 USD
+Total Rewards
+At Samsara, we build for the people who keep the global economy moving. We want owners, not passengers, which is why our rewards are designed to fuel high-impact builders. Our compensation program delivers above-market total compensation through a combination of base salary, performance-based bonus/variable pay, and equity (for eligible roles) in a high-growth public company. We meaningfully differentiate pay for our top performers, who have the opportunity to earn above-market compensation that can outpace the broader market over time.
+Beyond compensation, we provide the foundations that enable long-term success: a flexible, employee-led remote model, a professional development stipend, comprehensive health and parental leave plans, and more. If you’re ready to build for the long term and own the outcome, your journey starts here.
+Flexible Working 
+At Samsara, we embrace a flexible working model that caters to the diverse needs of our teams. Our offices are open for those who prefer to work in-person and we also support remote work where it aligns with our operational requirements. For certain positions, being close to one of our offices or within a specific geographic area is important to facilitate collaboration, access to resources, or alignment with our service regions. In these cases, the job description will clearly indicate any working location requirements. Our goal is to ensure that all members of our team can contribute effectively, whether they are working on-site, in a hybrid model, or fully remotely. All offers of employment are contingent upon an individual’s ability to secure and maintain the legal right to work at the company and in the specified work location, if applicable.
+Belonging at Samsara
+At Samsara, we welcome everyone regardless of their background. All qualified applicants will receive consideration for employment without regard to race, color, religion, national origin, sex, gender, gender identity, sexual orientation, protected veteran status, disability, age, and other characteristics protected by law. We depend on the unique approaches of our team members to help us solve complex problems and want to ensure that Samsara is a place where people from all backgrounds can make an impact.
+Accommodations 
+Samsara is an inclusive work environment, and we are committed to ensuring equal opportunity in employment for qualified persons with disabilities. Please email accessibleinterviewing@samsara.com or click here if you require any reasonable accommodations throughout the recruiting process.
+Our Commitment to Authenticity
+We use Tofu, a fraud detection tool, to validate the authenticity of applications and protect against identity fraud. This ensures we are connecting with real people and allows us to prioritize genuine candidates. Please see Samsara’s Candidate Privacy Notice for more information.
+Fraudulent Employment Offers
+Samsara is aware of scams involving fake job interviews and offers. Please know we do not charge fees to applicants at any stage of the hiring process. Official communication about your application will only come from emails ending in @samsara.com, @us-greenhouse-mail.io or @mail3.guide.co. For more information regarding fraudulent employment offers, please visit our blog post here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Pinterest</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Staff Software Engineer, Infrastructure Data Engineering</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY, US; Remote, US</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>remote</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pinterestcareers.com/jobs/?gh_jid=8162539</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.pinterestcareers.com/jobs/?gh_jid=8162539</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 23:50</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>open (live company feed)</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>About Pinterest:
+Millions of people around the world come to our platform to find creative ideas, dream about new possibilities and plan for memories that will last a lifetime. At Pinterest, we’re on a mission to bring everyone the inspiration to create a life they love, and that starts with the people behind the product.
+Discover a career where you ignite innovation for millions, transform passion into growth opportunities, celebrate each other’s unique experiences and embrace the flexibility to do your best work. Creating a career you love? It’s Possible.
+At Pinterest, AI isn't just a feature, it's a powerful partner that augments our creativity and amplifies our impact, and we’re looking for candidates who are excited to be a part of that. To get a complete picture of your experience and abilities, we’ll explore your foundational skills and how you collaborate with AI.
+Through our interview process, what matters most is that you can always explain your approach, showing us not just what you know, but how you think. You can read more about our AI interview philosophy and how we use AI in our recruiting process here.
+Pinterest is seeking a Staff Software Engineer to build the data systems that help teams understand and manage infrastructure usage and cost. You’ll lead the design and hands-on delivery of reliable data products, including pipelines, models, and services, that support infrastructure planning, cost attribution, and budget workflows. In this individual-contributor role, you’ll shape technical direction, navigate complex cross-team work, and make infrastructure data more accurate, consistent, and useful.
+What you’ll do:
+- Set technical direction and help define a roadmap for reliable, scalable infrastructure data products
+- Design, build, and operate production ingestion and transformation pipelines, data models, and services for infrastructure usage, cost, ownership, and planning
+- Strengthen shared data products with clear contracts, automated quality checks, reconciliation, documentation, and operational monitoring
+- Lead ambiguous, cross-functional initiatives from problem definition and technical trade-offs through rollout and adoption; raise the engineering bar through mentorship and design reviews
+- Leverage AI to scale the impact of yourself and the team, including:
+- Accelerate investigation of data-quality or pipeline issues while validating findings against source data and production evidence
+- Speed up implementation and documentation of data transformations and interfaces while testing and reviewing the results
+- Explore ways to help partners self-serve trusted infrastructure insights, protecting sensitive information and verifying outputs
+What we’re looking for:
+- Bachelor’s degree in computer science, a related field, or equivalent practical experience
+- Significant experience designing, building, and operating production data systems or data-intensive services at scale
+- Strong software engineering skills in Python and SQL, with a record of writing tested, maintainable production code
+- Deep experience with ingestion, large-scale ETL and transformation, data modeling, and workflow orchestration
+- Experience designing data interfaces and contracts and improving quality, freshness, completeness, and consistency
+- A track record of leading complex technical work across teams, from framing ambiguous problems to delivery and operation
+- Ability to influence through technical judgment and clear communication and to mentor other engineers
+- Experience operating dependable data pipelines or services, including testing, monitoring, and incident response
+- Experience with AWS or similar cloud environments
+- Demonstrated ability to use AI to improve speed and quality in your day-to-day workflow for relevant outputs
+- Strong track record of critical evaluation and verification of AI-assisted work (e.g., testing, source-checking, data validation, peer review)
+- High integrity and ownership: you protect sensitive data, avoid over-reliance on AI, and remain accountable for final decisions and deliverables
+- Bonus points for the following:
+- Experience with infrastructure cost or usage data, budgeting, shared data platforms, dbt, data lineage, or modeling hierarchical ownership
+- Hands-on experience with large, cloud-native multi-tenant platforms at Internet scale
+In-Office Requirement Statement: 
+- We recognize that the ideal environment for work is situational and may differ across departments. What this looks like day-to-day can vary based on the needs of each organization or role.
+- This role will need to be in the office for in-person collaboration 1-2 times/month and therefore can be situated anywhere in the country. 
+Relocation Statement:
+- This position is not eligible for relocation assistance. Visit our PinFlex page to learn more about our working model.
+#LI-REMOTE
+#LI-JT1
+At Pinterest we believe the workplace should be equitable, inclusive, and inspiring for every employee. In an effort to provide greater transparency, we are sharing the base salary range for this position. The position is also eligible for equity. Final salary is based on a number of factors including location, travel, relevant prior experience, or particular skills and expertise.
+Information regarding the culture at Pinterest and benefits available for this position can be found here.
+US based applicants only
+$177,185—$364,795 USD
+Our Commitment to Inclusion:
+Pinterest is an equal opportunity employer and makes employment decisions on the basis of merit. We want to have the best qualified people in every job. All qualified applicants will receive consideration for employment without regard to race, color, ancestry, national origin, religion or religious creed, sex (including pregnancy, childbirth, or related medical conditions), sexual orientation, gender, gender identity, gender expression, age, marital status, status as a protected veteran, physical or mental disability, medical condition, genetic information or characteristics (or those of a family member) or any other consideration made unlawful by applicable federal, state or local laws. We also consider qualified applicants regardless of criminal histories, consistent with legal requirements. If you require a medical or religious accommodation during the job application process, please complete this form for support.
+By submitting this application, I certify that all information submitted in my application and throughout the hiring process is true, accurate, and complete to the best of my knowledge. I understand that any false statement, omission, or misrepresentation may disqualify me from employment consideration or result in termination if discovered after hire.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P1"/>
+  <autoFilter ref="A1:P3"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -627,7 +874,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-25 18:45:39</t>
+          <t>2026-10-25 22:23:03</t>
         </is>
       </c>
     </row>
@@ -639,7 +886,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-26 00:15:39</t>
+          <t>2026-10-26 03:53:03</t>
         </is>
       </c>
     </row>
@@ -651,7 +898,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>168</t>
         </is>
       </c>
     </row>
@@ -663,7 +910,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -699,7 +946,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -723,7 +970,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: job feed run 2026-10-26 02:12 UTC
</commit_message>
<xml_diff>
--- a/output/DataEngineerJobs_2026-10-26.xlsx
+++ b/output/DataEngineerJobs_2026-10-26.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Run Log" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Jobs'!$A$1:$P$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Jobs'!$A$1:$P$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Excluded'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,10 +33,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <color rgb="001155CC"/>
-      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -64,16 +60,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -440,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -543,245 +533,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Samsara</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Senior AI Data &amp; Analytics Engineer II</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Remote - Seattle</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>remote</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Full-time</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.samsara.com/company/careers/roles/8302004?gh_jid=8302004</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>accessibleinterviewing@samsara.com</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.samsara.com/company/careers/roles/8302004?gh_jid=8302004</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>5yr</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-20 02:25</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>greenhouse</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>open (live company feed)</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>Who we are
-Samsara (NYSE: IOT) is the pioneer of the Connected Operations™ Cloud, which is a platform that enables organizations that depend on physical operations to harness Internet of Things (IoT) data to develop actionable insights and improve their operations. At Samsara, we are helping improve the safety, efficiency and sustainability of the physical operations that power our global economy. Representing more than 40% of global GDP, these industries are the infrastructure of our planet, including agriculture, construction, field services, transportation, and manufacturing — and we are excited to help digitally transform their operations at scale.
-Working at Samsara means you’ll help define the future of physical operations and be on a team that’s shaping an exciting array of product solutions, including Video-Based Safety, Vehicle Telematics, Apps and Driver Workflows, and Equipment Monitoring. As part of a recently public company, you’ll have the autonomy and support to make an impact as we build for the long term.
-About the role:
-Want to build the data foundation powering AI and self-serve analytics at scale? As part of Samsara's Marketing Data and Analytics (MDA) Engineering team, you will shape the technical roadmap alongside our BI and Data Science peers. You will architect core Databricks pipelines, Gold Layer tables, and semantic models, turning ambitious, ambiguous business challenges into high-value data products, autonomous agents, and cross-functional automation.
-This role is open to candidates residing in the US.
-You should apply if:
-- You want to impact the industries that run our world: Your efforts will result in real-world impact – helping to keep the lights on, get food into grocery stores, reduce emissions, and most importantly, ensure workers return home safely.
-- You are the architect of your own career: If you put in the work, this role won’t be your last at Samsara. We set up our employees for success and have built a culture that encourages rapid career development, countless opportunities to experiment and master your craft in a hyper growth environment.
-- You’re energized by our opportunity: The vision we have to digitize large sectors of the global economy requires your full focus and best efforts to bring forth creative, ambitious ideas for our customers.
-- You want to be with the best: At Samsara, we win together, celebrate together and support each other. You will be surrounded by a high-calibre team that will encourage you to do your best. 
-In this role, you will:
-- Partner on defining the strategy and multi-quarter roadmap for MDA's data and AI foundation.
-- Architect and own Samsara's marketing data infrastructure: ETL/ELT pipelines, Databricks Gold Layer tables, and the core data models that power segmentation, targeting, automation, and analytics.
-- Design the semantic layers, data dictionaries, and structured documentation that enable self-serve BI and conversational analytics, partnering with the BI team to ensure core sales and marketing KPIs are built on trusted, well-modeled data.
-- Translate ambiguous business questions from Marketing, Sales, and R&amp;D into clear requirements and scalable solutions, working autonomously without dedicated PM support and influencing decisions with data and sound reasoning.
-- Lead complex, cross-team initiatives end to end: stand up new data pipelines and integrations quickly, manage risk across interdependent teams, and own the reliability and data quality of what ships.
-- Serve as the senior technical lead for the team's hardest problems: raise the bar for engineering quality and code review, remove bottlenecks that slow multiple teams, and mentor engineers and analysts. 
-- Drive the strategic use of AI to solve ambiguous, high-impact problems: build AI-enabled data products and agents, with the integrations, retrieval pipelines, and evaluation practices that keep them reliable and trustworthy.
-- Identify and automate manual workflows with AI across Marketing and GTM teams, taking ideas from concept to prototype to production and influencing org roadmaps.
-- Ship high-quality Python and SQL, increasingly by directing agentic coding tools, while holding a high bar for reviewing and verifying AI-generated work before it reaches production.
-- Champion, role model, and embed Samsara’s cultural principles (Focus on Customer Success, Build for the Long Term, Adopt a Growth Mindset, Be Inclusive, Win as a Team) as we scale globally and across new offices.
-Minimum requirements for the role:
-- 8+ years of experience in data engineering, analytics engineering, or AI engineering, including deep hands-on data engineering experience.
-- Expert-level Python and SQL, with strong hands-on data modeling and DBT experience.
-- Deep experience with data warehouse and lakehouse architectures, ETL/ELT, and the modern data stack, including hands-on Databricks (or similar, such as Snowflake or BigQuery).
-- Experience building semantic layers and structured documentation optimized for AI ingestion and agentic workflows.
-- Agentic coding tools (e.g., Claude Code, Cursor) are part of your regular workflow, and you verify and take ownership of AI-generated output.
-- Experience building, shipping, evaluating, and monitoring LLM or agent systems in production.
-- Track record of leading complex, cross-team data initiatives, including independent requirements gathering with technical and non-technical stakeholders.
-- Experience supporting Marketing, Sales, or Product teams.
-An ideal candidate also has:
-- Experience working with Databricks and building AI Agents within the ecosystem. 
-- Software engineering background beyond data or AI engineering, with a track record of turning ambiguous, unfamiliar problems into well-architected, delivered solutions.
-- Expertise in data visualization and building dashboards for sales and marketing KPIs.
-- Familiarity with go-to-market data and systems: CRM (e.g., Salesforce), marketing automation, web analytics, and MarTech tools.
-- Experience building interactive applications with Streamlit, Claude workflows, or web frameworks.
-- Data science, machine learning, or predictive analytics experience.
-- Comfort working in an exploratory environment, testing and iterating on new data sources and methodologies.
-The compensation range shown spans approved pay zones for this role. Your primary work location determines the range applicable to you, which may be narrower than the full range displayed.
-The range of annual base salary for full-time employees for this position is below. Please note that base pay offered may vary depending on factors including your city of residence, job-related knowledge, skills, and experience. This role is also eligible for an initial RSU grant with no vesting cliff, and ongoing refresh opportunities tied to performance, subject to plan terms and conditions. Learn more about our total rewards and benefits below.
-Annual Base Salary
-$137,445—$231,000 USD
-Total Rewards
-At Samsara, we build for the people who keep the global economy moving. We want owners, not passengers, which is why our rewards are designed to fuel high-impact builders. Our compensation program delivers above-market total compensation through a combination of base salary, performance-based bonus/variable pay, and equity (for eligible roles) in a high-growth public company. We meaningfully differentiate pay for our top performers, who have the opportunity to earn above-market compensation that can outpace the broader market over time.
-Beyond compensation, we provide the foundations that enable long-term success: a flexible, employee-led remote model, a professional development stipend, comprehensive health and parental leave plans, and more. If you’re ready to build for the long term and own the outcome, your journey starts here.
-Flexible Working 
-At Samsara, we embrace a flexible working model that caters to the diverse needs of our teams. Our offices are open for those who prefer to work in-person and we also support remote work where it aligns with our operational requirements. For certain positions, being close to one of our offices or within a specific geographic area is important to facilitate collaboration, access to resources, or alignment with our service regions. In these cases, the job description will clearly indicate any working location requirements. Our goal is to ensure that all members of our team can contribute effectively, whether they are working on-site, in a hybrid model, or fully remotely. All offers of employment are contingent upon an individual’s ability to secure and maintain the legal right to work at the company and in the specified work location, if applicable.
-Belonging at Samsara
-At Samsara, we welcome everyone regardless of their background. All qualified applicants will receive consideration for employment without regard to race, color, religion, national origin, sex, gender, gender identity, sexual orientation, protected veteran status, disability, age, and other characteristics protected by law. We depend on the unique approaches of our team members to help us solve complex problems and want to ensure that Samsara is a place where people from all backgrounds can make an impact.
-Accommodations 
-Samsara is an inclusive work environment, and we are committed to ensuring equal opportunity in employment for qualified persons with disabilities. Please email accessibleinterviewing@samsara.com or click here if you require any reasonable accommodations throughout the recruiting process.
-Our Commitment to Authenticity
-We use Tofu, a fraud detection tool, to validate the authenticity of applications and protect against identity fraud. This ensures we are connecting with real people and allows us to prioritize genuine candidates. Please see Samsara’s Candidate Privacy Notice for more information.
-Fraudulent Employment Offers
-Samsara is aware of scams involving fake job interviews and offers. Please know we do not charge fees to applicants at any stage of the hiring process. Official communication about your application will only come from emails ending in @samsara.com, @us-greenhouse-mail.io or @mail3.guide.co. For more information regarding fraudulent employment offers, please visit our blog post here.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Pinterest</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Staff Software Engineer, Infrastructure Data Engineering</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>New York, NY, US; Remote, US</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>remote</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Full-time</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.pinterestcareers.com/jobs/?gh_jid=8162539</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.pinterestcareers.com/jobs/?gh_jid=8162539</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-19 23:50</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>greenhouse</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr"/>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>open (live company feed)</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>About Pinterest:
-Millions of people around the world come to our platform to find creative ideas, dream about new possibilities and plan for memories that will last a lifetime. At Pinterest, we’re on a mission to bring everyone the inspiration to create a life they love, and that starts with the people behind the product.
-Discover a career where you ignite innovation for millions, transform passion into growth opportunities, celebrate each other’s unique experiences and embrace the flexibility to do your best work. Creating a career you love? It’s Possible.
-At Pinterest, AI isn't just a feature, it's a powerful partner that augments our creativity and amplifies our impact, and we’re looking for candidates who are excited to be a part of that. To get a complete picture of your experience and abilities, we’ll explore your foundational skills and how you collaborate with AI.
-Through our interview process, what matters most is that you can always explain your approach, showing us not just what you know, but how you think. You can read more about our AI interview philosophy and how we use AI in our recruiting process here.
-Pinterest is seeking a Staff Software Engineer to build the data systems that help teams understand and manage infrastructure usage and cost. You’ll lead the design and hands-on delivery of reliable data products, including pipelines, models, and services, that support infrastructure planning, cost attribution, and budget workflows. In this individual-contributor role, you’ll shape technical direction, navigate complex cross-team work, and make infrastructure data more accurate, consistent, and useful.
-What you’ll do:
-- Set technical direction and help define a roadmap for reliable, scalable infrastructure data products
-- Design, build, and operate production ingestion and transformation pipelines, data models, and services for infrastructure usage, cost, ownership, and planning
-- Strengthen shared data products with clear contracts, automated quality checks, reconciliation, documentation, and operational monitoring
-- Lead ambiguous, cross-functional initiatives from problem definition and technical trade-offs through rollout and adoption; raise the engineering bar through mentorship and design reviews
-- Leverage AI to scale the impact of yourself and the team, including:
-- Accelerate investigation of data-quality or pipeline issues while validating findings against source data and production evidence
-- Speed up implementation and documentation of data transformations and interfaces while testing and reviewing the results
-- Explore ways to help partners self-serve trusted infrastructure insights, protecting sensitive information and verifying outputs
-What we’re looking for:
-- Bachelor’s degree in computer science, a related field, or equivalent practical experience
-- Significant experience designing, building, and operating production data systems or data-intensive services at scale
-- Strong software engineering skills in Python and SQL, with a record of writing tested, maintainable production code
-- Deep experience with ingestion, large-scale ETL and transformation, data modeling, and workflow orchestration
-- Experience designing data interfaces and contracts and improving quality, freshness, completeness, and consistency
-- A track record of leading complex technical work across teams, from framing ambiguous problems to delivery and operation
-- Ability to influence through technical judgment and clear communication and to mentor other engineers
-- Experience operating dependable data pipelines or services, including testing, monitoring, and incident response
-- Experience with AWS or similar cloud environments
-- Demonstrated ability to use AI to improve speed and quality in your day-to-day workflow for relevant outputs
-- Strong track record of critical evaluation and verification of AI-assisted work (e.g., testing, source-checking, data validation, peer review)
-- High integrity and ownership: you protect sensitive data, avoid over-reliance on AI, and remain accountable for final decisions and deliverables
-- Bonus points for the following:
-- Experience with infrastructure cost or usage data, budgeting, shared data platforms, dbt, data lineage, or modeling hierarchical ownership
-- Hands-on experience with large, cloud-native multi-tenant platforms at Internet scale
-In-Office Requirement Statement: 
-- We recognize that the ideal environment for work is situational and may differ across departments. What this looks like day-to-day can vary based on the needs of each organization or role.
-- This role will need to be in the office for in-person collaboration 1-2 times/month and therefore can be situated anywhere in the country. 
-Relocation Statement:
-- This position is not eligible for relocation assistance. Visit our PinFlex page to learn more about our working model.
-#LI-REMOTE
-#LI-JT1
-At Pinterest we believe the workplace should be equitable, inclusive, and inspiring for every employee. In an effort to provide greater transparency, we are sharing the base salary range for this position. The position is also eligible for equity. Final salary is based on a number of factors including location, travel, relevant prior experience, or particular skills and expertise.
-Information regarding the culture at Pinterest and benefits available for this position can be found here.
-US based applicants only
-$177,185—$364,795 USD
-Our Commitment to Inclusion:
-Pinterest is an equal opportunity employer and makes employment decisions on the basis of merit. We want to have the best qualified people in every job. All qualified applicants will receive consideration for employment without regard to race, color, ancestry, national origin, religion or religious creed, sex (including pregnancy, childbirth, or related medical conditions), sexual orientation, gender, gender identity, gender expression, age, marital status, status as a protected veteran, physical or mental disability, medical condition, genetic information or characteristics (or those of a family member) or any other consideration made unlawful by applicable federal, state or local laws. We also consider qualified applicants regardless of criminal histories, consistent with legal requirements. If you require a medical or religious accommodation during the job application process, please complete this form for support.
-By submitting this application, I certify that all information submitted in my application and throughout the hiring process is true, accurate, and complete to the best of my knowledge. I understand that any false statement, omission, or misrepresentation may disqualify me from employment consideration or result in termination if discovered after hire.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:P3"/>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
-  </hyperlinks>
+  <autoFilter ref="A1:P1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -874,7 +627,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-25 22:23:03</t>
+          <t>2026-10-26 02:11:12</t>
         </is>
       </c>
     </row>
@@ -886,7 +639,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-26 03:53:03</t>
+          <t>2026-10-26 07:41:12</t>
         </is>
       </c>
     </row>
@@ -946,7 +699,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -970,7 +723,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
     </row>

</xml_diff>